<commit_message>
Govern DDUP model configuration and backlog tier matching
</commit_message>
<xml_diff>
--- a/docs/03_backlog.xlsx
+++ b/docs/03_backlog.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="27040" windowHeight="15320" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Backlog" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Epics" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Legend" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backlog'!$A$1:$I$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backlog'!$A$1:$I$150</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I148"/>
+  <dimension ref="A1:I150"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7581,8 +7581,112 @@
         </is>
       </c>
     </row>
+    <row r="149" ht="112" customHeight="1">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>US-149</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>15. Deduplication &amp; Record Matching</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>DAT-DDUP</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>System Admin / DQA Approver</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>As a System Administrator, I want a governed Tier 2 exact-phone matching model, so that normalised phone matches can be reviewed without code-defined matching policy.</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>- Uses the canonical derived field telephone_1_e164 and the approved DDUP configuration only
+- No comparison field, score, queue threshold, or matching reason is supplied by application code
+- Draft model validates against the Questionnaire/Data Dictionary and derived-field registry before submission
+- A different authorised approver activates the version; the preceding active version is retained and auditable
+- Discovery, DIH candidate screening, and the DDUP queue consume the same approved model version
+- Regression tests cover disabled, valid, unregistered-field, and approval-separation cases</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>DDUP configuration SSOT; Questionnaire Authoring Data Dictionary; ADR-0001</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Blocked until the phone-normalisation contract and policy values are approved. Tier 2 must begin disabled; do not introduce code defaults.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="112" customHeight="1">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>US-150</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>15. Deduplication &amp; Record Matching</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>DAT-DDUP</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>System Admin / DQA Approver / DPO</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>As a System Administrator and DPO, I want a governed Tier 3 probabilistic matching model, so that calibrated candidate matching can be introduced only through an approved, auditable model version.</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>- Features, comparators, weights, blocking field, review threshold, and any auto-merge policy come solely from the approved DDUP configuration
+- Every configured field must resolve through the Questionnaire/Data Dictionary or declared derived-field registry
+- Calibration evidence, DPO review, and independent approval are recorded before activation
+- Disabled or incomplete Tier 3 configuration produces no candidates; there is no fallback score, threshold, or weight in application code
+- Queue results retain model version and feature trace for review and reproducibility
+- Regression tests cover schema validation, calibration boundaries from configuration, approval separation, and DIH/DDUP shared-model propagation</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>DDUP configuration SSOT; Questionnaire Authoring Data Dictionary; PMT/DQA/DIH integration; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Blocked until comparison-comparator registry, calibration dataset, governance policy, and DPO approval exist. No auto-merge policy may be inferred.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I75"/>
+  <autoFilter ref="A1:I150"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7982,13 +8086,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D16" t="n">
         <v>5</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>

</xml_diff>